<commit_message>
Auto update (2026-04-30 08:52:04) | Files: node/AlarmReport.xlsx vswr/AlarmReport.xlsx
</commit_message>
<xml_diff>
--- a/vswr/AlarmReport.xlsx
+++ b/vswr/AlarmReport.xlsx
@@ -166,12 +166,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28 23:37:45</t>
+          <t>2026-04-29 23:29:14</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28 23:37:45</t>
+          <t>2026-04-29 23:29:14</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -193,32 +193,32 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>PRIKRO</t>
+          <t>MASSIMBA</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AC901</t>
+          <t>AC172</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>PRIKRO</t>
+          <t>BB_AC172_GL</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Board Temperature Unacceptable</t>
+          <t>Critical Temperature Performance Degraded</t>
         </is>
       </c>
       <c r="G3" s="2"/>
@@ -229,12 +229,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 01:41:43</t>
+          <t>2026-04-29 13:02:39</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 01:41:43</t>
+          <t>2026-04-29 23:57:33</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -244,39 +244,39 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=0, Slot No.=3, Board Type=UBBP, Current Board Temperature (C/F)=95/203, Specific Problem=Temperature too High</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC172_GL,ManagedElement=BB_AC172_GL,Equipment=1,FieldReplaceableUnit=RRUS-11_B8 2502170920</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>LOULOUDOU</t>
+          <t>MASSIMBA</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>AC774</t>
+          <t>AC172</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>BB_AC774_GL</t>
+          <t>BB_AC172_W</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -292,12 +292,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23 11:02:45</t>
+          <t>2026-04-29 13:02:39</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-04-23 11:02:45</t>
+          <t>2026-04-29 23:57:33</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -307,7 +307,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC774_GL,ManagedElement=BB_AC774_GL,Equipment=1,FieldReplaceableUnit=RRU-6_B3 2497805831</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_RadioNode,MeContext=BB_AC172_W,ManagedElement=BB_AC172_W,Equipment=1,FieldReplaceableUnit=RRUS-5 2502189151</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -355,12 +355,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28 22:03:07</t>
+          <t>2026-04-29 23:11:24</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:55:44</t>
+          <t>2026-04-29 23:11:24</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -370,7 +370,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_RadioNode,MeContext=BB_AC172_W,ManagedElement=BB_AC172_W,Equipment=1,FieldReplaceableUnit=RRUS-5 2501830907</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_RadioNode,MeContext=BB_AC172_W,ManagedElement=BB_AC172_W,Equipment=1,FieldReplaceableUnit=RRUS-4 2501141387</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -418,12 +418,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28 22:03:07</t>
+          <t>2026-04-29 23:11:24</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:55:44</t>
+          <t>2026-04-29 23:11:24</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -433,7 +433,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC172_GL,ManagedElement=BB_AC172_GL,Equipment=1,FieldReplaceableUnit=RRUS-11_B8 2501830908</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC172_GL,ManagedElement=BB_AC172_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2501141386</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -450,12 +450,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>MASSIMBA</t>
+          <t>NDOTRE</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AC172</t>
+          <t>AC372</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -465,7 +465,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>BB_AC172_W</t>
+          <t>BB_AC372_W</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -481,12 +481,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:58:30</t>
+          <t>2026-04-29 23:39:20</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:58:30</t>
+          <t>2026-04-29 23:56:56</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -496,7 +496,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_RadioNode,MeContext=BB_AC172_W,ManagedElement=BB_AC172_W,Equipment=1,FieldReplaceableUnit=RRUS-4 2501141387</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC06,SubNetwork=AORNC06_RadioNode,MeContext=BB_AC372_W,ManagedElement=BB_AC372_W,Equipment=1,FieldReplaceableUnit=PSU-1 2502224640</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -513,27 +513,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>MASSIMBA</t>
+          <t>NDOTRE</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>AC172</t>
+          <t>AC372</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>BB_AC172_GL</t>
+          <t>BB_AC372_W</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Critical Temperature Performance Degraded</t>
+          <t>Critical Temperature Taken Out of Service</t>
         </is>
       </c>
       <c r="G8" s="2"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:58:30</t>
+          <t>2026-04-29 22:46:52</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:58:30</t>
+          <t>2026-04-29 23:34:02</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC172_GL,ManagedElement=BB_AC172_GL,Equipment=1,FieldReplaceableUnit=RRUS-10_B8 2501141386</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC06,SubNetwork=AORNC06_RadioNode,MeContext=BB_AC372_W,ManagedElement=BB_AC372_W,Equipment=1,FieldReplaceableUnit=PSU-2 2502189370</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:51:03</t>
+          <t>2026-04-29 23:23:07</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:51:03</t>
+          <t>2026-04-29 23:23:07</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC06,SubNetwork=AORNC06_RadioNode,MeContext=BB_AC372_W,ManagedElement=BB_AC372_W,Equipment=1,FieldReplaceableUnit=1 2501305121</t>
+          <t>SubNetwork=RNC,SubNetwork=AORNC06,SubNetwork=AORNC06_RadioNode,MeContext=BB_AC372_W,ManagedElement=BB_AC372_W,Equipment=1,FieldReplaceableUnit=1 2502210194</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -733,12 +733,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:32:23</t>
+          <t>2026-04-29 23:43:30</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:32:23</t>
+          <t>2026-04-29 23:43:30</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -760,48 +760,48 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>KORHOGO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>TAFIRE</t>
+          <t>NASSIAN</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>AC253</t>
+          <t>AC546</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>AC253</t>
+          <t>WAC546</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>RF Unit Temperature Unacceptable</t>
+          <t>NTP Server Reachability Fault</t>
         </is>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 14:26:33</t>
+          <t>2026-04-29 23:36:51</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 14:26:33</t>
+          <t>2026-04-29 23:57:33</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -811,60 +811,60 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Cabinet No.=1, Subrack No.=4, Slot No.=0, Board Type=MRFU, PA Temperature ( C/F)=91/196, Board Temperature ( C/F)=83/181, Output Power (0.1 dBm)=469, Site No.=21, Site Type=BTS3900A GSM, Site Name=AC253</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC546,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=7 2502442786</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>KORHOGO</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>TAFIRE</t>
+          <t>NASSIAN</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>AC253</t>
+          <t>AC546</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>3G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>TAFIRE</t>
+          <t>WAC546</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>RF Unit Temperature Unacceptable</t>
+          <t>NTP Server Reachability Fault</t>
         </is>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 14:26:34</t>
+          <t>2026-04-29 23:51:45</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 14:26:34</t>
+          <t>2026-04-29 23:57:32</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -874,39 +874,39 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Cabinet No.=1, Subrack No.=4, Slot No.=0, Board Type=MRFU, PA Temperature (C/F)=91/196, Board Temperature(C/F)=83/181, Output Power (0.1 dBm)=469</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_GROUP,MeContext=WAC546,ManagedElement=1,IpSystem=1,IpAccessHostEt=1,IpSyncRef=8 2502442785</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>KORHOGO</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>NIEKEIDE</t>
+          <t>TAFIRE</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>AC872</t>
+          <t>AC253</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2G,3G,4G</t>
+          <t>2G</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>NIEKEIDE</t>
+          <t>AC253</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -922,12 +922,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26 07:25:16</t>
+          <t>2026-04-22 14:26:33</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26 07:25:16</t>
+          <t>2026-04-22 14:26:33</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Cabinet No.=0, Subrack No.=4, Slot No.=0, Board Type=MRFU, PA Temperature (C/F)=91/196, Board Temperature(C/F)=83/181, Output Power (0.1 dBm)=30</t>
+          <t>Cabinet No.=1, Subrack No.=4, Slot No.=0, Board Type=MRFU, PA Temperature ( C/F)=91/196, Board Temperature ( C/F)=83/181, Output Power (0.1 dBm)=469, Site No.=21, Site Type=BTS3900A GSM, Site Name=AC253</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -949,48 +949,48 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>KORHOGO</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>TAFIRE</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC253</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G,4G</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>BB_AC534_GL</t>
+          <t>TAFIRE</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RF Unit Temperature Unacceptable</t>
         </is>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27 13:41:14</t>
+          <t>2026-04-22 14:26:34</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27 13:41:14</t>
+          <t>2026-04-22 14:26:34</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1000,60 +1000,60 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC534_GL,ManagedElement=BB_AC534_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2501142422</t>
+          <t>Cabinet No.=1, Subrack No.=4, Slot No.=0, Board Type=MRFU, PA Temperature (C/F)=91/196, Board Temperature(C/F)=83/181, Output Power (0.1 dBm)=469</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>BOUBOURY</t>
+          <t>MAMINIGUI</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>AC534</t>
+          <t>AC868</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>BB_AC534_GL</t>
+          <t>MAMINIGUI</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RF Unit Temperature Unacceptable</t>
         </is>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27 13:41:19</t>
+          <t>2026-04-29 20:54:42</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2026-04-27 13:41:19</t>
+          <t>2026-04-29 20:54:42</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1063,60 +1063,60 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC534_GL,ManagedElement=BB_AC534_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2501146219</t>
+          <t>Cabinet No.=0, Subrack No.=4, Slot No.=2, Board Type=MRFU, PA Temperature (C/F)=91/196, Board Temperature(C/F)=86/187, Output Power (0.1 dBm)=465</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>LAOGUIE</t>
+          <t>NIEKEIDE</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>AC278</t>
+          <t>AC872</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,3G,4G</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>BB_AC278_W</t>
+          <t>NIEKEIDE</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sync Frequency Reference Not Reliable</t>
+          <t>RF Unit Temperature Unacceptable</t>
         </is>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Information</t>
+          <t>Minor</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 22:02:16</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 22:02:16</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1126,39 +1126,39 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_RadioNode,MeContext=BB_AC278_W,ManagedElement=BB_AC278_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2502012465</t>
+          <t>Cabinet No.=0, Subrack No.=4, Slot No.=0, Board Type=MRFU, PA Temperature (C/F)=91/196, Board Temperature(C/F)=83/181, Output Power (0.1 dBm)=443</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>LAOGUIE</t>
+          <t>SAYE</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>AC278</t>
+          <t>ET450</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>BB_AC278_GL</t>
+          <t>BB_ET450_W</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 21:58:45</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 21:58:45</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC278_GL,ManagedElement=BB_AC278_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2502012461</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_ET450_W,ManagedElement=BB_ET450_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2502425049</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1201,17 +1201,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>LAOGUIE</t>
+          <t>SAYE</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>AC278</t>
+          <t>ET450</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>BB_AC278_W</t>
+          <t>BB_ET450_W</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 21:58:45</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 21:58:45</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=AORNC09,SubNetwork=AORNC09_RadioNode,MeContext=BB_AC278_W,ManagedElement=BB_AC278_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2502012464</t>
+          <t>SubNetwork=RNC,SubNetwork=AGRNC22,SubNetwork=AGRNC22_RadioNode,MeContext=BB_ET450_W,ManagedElement=BB_ET450_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2502425050</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1264,17 +1264,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>LAOGUIE</t>
+          <t>GROBIASSOUME</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>AC278</t>
+          <t>AC964</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>BB_AC278_GL</t>
+          <t>BB_AC964_GL</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1300,12 +1300,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 22:57:22</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:47:07</t>
+          <t>2026-04-29 22:57:22</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC278_GL,ManagedElement=BB_AC278_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2502012463</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC964_GL,ManagedElement=BB_AC964_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2502364630</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -1327,48 +1327,48 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>DJOUROUTOU</t>
+          <t>GROBIASSOUME</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>AC787</t>
+          <t>AC964</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>WAC787</t>
+          <t>BB_AC964_GL</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:33:58</t>
+          <t>2026-04-29 22:57:22</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:33:58</t>
+          <t>2026-04-29 22:57:22</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WAC787,ManagedElement=1,TransportNetwork=1,Synchronization=1 2501830020</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC964_GL,ManagedElement=BB_AC964_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2502364629</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -1390,48 +1390,48 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>GBAPET</t>
+          <t>GROBIASSOUME</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>AC781</t>
+          <t>AC964</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>LAC781</t>
+          <t>BB_AC964_W</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:37:11</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:37:11</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=EnodeB,MeContext=LAC781,ManagedElement=1,TransportNetwork=1,Synchronization=1 2501848401</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_AC964_W,ManagedElement=BB_AC964_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2502355932</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -1453,48 +1453,48 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>PARA</t>
+          <t>GUIGUEDOU</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>ET178</t>
+          <t>AC776</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>WET178</t>
+          <t>BB_AC776_GL</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sync Reference PDV Problem</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Major</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:52:53</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29 07:52:53</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2501838571</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC776_GL,ManagedElement=BB_AC776_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=1 2502335081</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -1516,48 +1516,48 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>NDOTRE</t>
+          <t>GROBIASSOUME</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>AC372</t>
+          <t>AC964</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>RAN</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>AC372-OSmon</t>
+          <t>BB_AC964_W</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Temperature Outside Limits</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26 17:36:30</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>2026-04-26 17:36:30</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=TCU,MeContext=AC372-OSmon,STN=0,Equipment=0 2500730363</t>
+          <t>SubNetwork=RNC,SubNetwork=SIRNC08,SubNetwork=SIRNC08_RadioNode,MeContext=BB_AC964_W,ManagedElement=BB_AC964_W,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2502355931</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -1579,48 +1579,48 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>EBIMPE</t>
+          <t>GUIGUEDOU</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>AC691</t>
+          <t>AC776</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ESC</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ESC_AC691_C6610</t>
+          <t>BB_AC776_GL</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Temperature Sensor Failure</t>
+          <t>Sync Frequency Reference Not Reliable</t>
         </is>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>2026-04-22 21:24:30</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>2026-04-25 09:24:17</t>
+          <t>2026-04-29 22:57:23</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=ESC,MeContext=ESC_AC691_C6610,ManagedElement=ESC_AC691_C6610,Equipment=1,FieldReplaceableUnit=PowerController,Sensor=1 2498913489</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC776_GL,ManagedElement=BB_AC776_GL,Transport=1,Synchronization=1,RadioEquipmentClock=1,RadioEquipmentClockReference=2 2502335080</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -1642,52 +1642,48 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>BB_ET833_GL</t>
+          <t>WET178</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
+          <t>Sync Reference PDV Problem</t>
+        </is>
+      </c>
+      <c r="G26" s="2"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Major</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 00:48:15</t>
+          <t>2026-04-29 21:55:05</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 00:48:15</t>
+          <t>2026-04-29 23:38:57</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -1697,7 +1693,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2499389965</t>
+          <t>SubNetwork=RNC,SubNetwork=YORNC02,SubNetwork=YORNC02_GROUP,MeContext=WET178,ManagedElement=1,TransportNetwork=1,Synchronization=1 2502224693</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -1709,52 +1705,48 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TIEVIESSOU</t>
+          <t>NDOTRE</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>ET833</t>
+          <t>AC372</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>BB_ET833_W</t>
+          <t>AC372-OSmon</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
+          <t>Temperature Outside Limits</t>
+        </is>
+      </c>
+      <c r="G27" s="2"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 00:48:15</t>
+          <t>2026-04-26 17:36:30</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 00:48:15</t>
+          <t>2026-04-26 17:36:30</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -1764,7 +1756,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,MeContext=BB_ET833_W,ManagedElement=BB_ET833_W,Equipment=1,FieldReplaceableUnit=RRU-2_B1,RfPort=B 2499389964</t>
+          <t>SubNetwork=TCU,MeContext=AC372-OSmon,STN=0,Equipment=0 2500730363</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -1776,39 +1768,35 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>GOUDI</t>
+          <t>EBIMPE</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>ET148</t>
+          <t>AC691</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>ESC</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>BB_ET148_GL</t>
+          <t>ESC_AC691_C6610</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
+          <t>Temperature Sensor Failure</t>
+        </is>
+      </c>
+      <c r="G28" s="2"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Minor</t>
@@ -1816,12 +1804,12 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 09:36:27</t>
+          <t>2026-04-22 21:24:30</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 09:36:27</t>
+          <t>2026-04-25 09:24:17</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -1831,7 +1819,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2499554416</t>
+          <t>SubNetwork=ESC,MeContext=ESC_AC691_C6610,ManagedElement=ESC_AC691_C6610,Equipment=1,FieldReplaceableUnit=PowerController,Sensor=1 2498913489</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -1843,52 +1831,48 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>SONGON_BEL_HORIZON</t>
+          <t>MASSARANA</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>ET815</t>
+          <t>AC011</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>2G,4G</t>
+          <t>RAN</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>BB_ET815_GL</t>
+          <t>AC011-OSmon</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>VSWR Over Threshold</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
+          <t>Temperature is near limits</t>
+        </is>
+      </c>
+      <c r="G29" s="2"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Information</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 22:18:05</t>
+          <t>2026-04-29 22:42:24</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 22:18:05</t>
+          <t>2026-04-29 22:42:24</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -1898,7 +1882,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET815_GL,ManagedElement=BB_ET815_GL,Equipment=1,FieldReplaceableUnit=RRUS-1_B8B20,RfPort=C 2497193771</t>
+          <t>SubNetwork=TCU,MeContext=AC011-OSmon,STN=0,Equipment=0 2502442793</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -1915,22 +1899,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>SONGON_BEL_HORIZON</t>
+          <t>TIEVIESSOU</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>ET815</t>
+          <t>ET833</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G,4G</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>BB_ET815_W</t>
+          <t>BB_ET833_GL</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1950,12 +1934,12 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 22:18:05</t>
+          <t>2026-04-24 00:48:15</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>2026-04-24 22:18:05</t>
+          <t>2026-04-24 00:48:15</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -1965,7 +1949,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>SubNetwork=RNC,SubNetwork=YORNC07,MeContext=BB_ET815_W,ManagedElement=BB_ET815_W,Equipment=1,FieldReplaceableUnit=RRU-4,RfPort=C 2497193772</t>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET833_GL,ManagedElement=BB_ET833_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=B 2499389965</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -1977,65 +1961,333 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>TIEVIESSOU</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>ET833</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>BB_ET833_W</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24 00:48:15</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24 00:48:15</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,MeContext=BB_ET833_W,ManagedElement=BB_ET833_W,Equipment=1,FieldReplaceableUnit=RRU-2_B1,RfPort=B 2499389964</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>GOUDI</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>ET148</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>BB_ET148_GL</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24 09:36:27</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-24 09:36:27</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_ET148_GL,ManagedElement=BB_ET148_GL,Equipment=1,FieldReplaceableUnit=RRUS-3_B1B3,RfPort=C 2499554416</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>ABIDJAN 04</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>OGHLWAPO</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>AC552</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>3G</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>BB_AC552_W</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>VSWR Over Threshold</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Minor</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-28 13:18:46</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>2026-04-28 13:18:46</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Uncleared</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:01:31</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:01:31</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>SubNetwork=RNC,SubNetwork=ABRNC03,SubNetwork=ABRNC03_RadioNode,MeContext=BB_AC552_W,ManagedElement=BB_AC552_W,Equipment=1,FieldReplaceableUnit=RRU-5,RfPort=A 2501642584</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>IROBO</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>AC522</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>3G</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>BB_AC522_W</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:33:30</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29 11:33:30</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>SubNetwork=RNC,SubNetwork=YORNC07,SubNetwork=YORNC07_RadioNode,MeContext=BB_AC522_W,ManagedElement=BB_AC522_W,Equipment=1,FieldReplaceableUnit=RRU-1,RfPort=A 2502118086</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>GAGNOA</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>DIVO_DIALOGUE</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>AC933</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2G,4G</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>BB_AC933_GL</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>VSWR Over Threshold</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:13:35</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-29 15:13:35</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Uncleared</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>SubNetwork=LTE_RadioNode,MeContext=BB_AC933_GL,ManagedElement=BB_AC933_GL,Equipment=1,FieldReplaceableUnit=RRUS-11_B8,RfPort=A 2500634589</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>ERICSSON</t>
         </is>

</xml_diff>